<commit_message>
Corrige le redimensionnement bloqué et la remontée des chiffres en Facture Propriétaire
- Autorise l'ajustement de la largeur des colonnes et de la hauteur des lignes
  malgré la protection des feuilles (formatColumns/formatRows n'étaient pas
  autorisés, empêchant tout redimensionnement).
- La liste des biens utilisée dans toutes les listes déroulantes et les
  formules de correspondance (Liste_Biens) pointe désormais directement sur
  les noms réels saisis dans l'onglet Biens (Biens!A5:A14) au lieu d'une
  liste figée "Bien 1"..."Bien 10" dans Paramètres. Auparavant, dès qu'un
  bien était renommé dans l'onglet Biens, les correspondances (taux de
  commission, coordonnées propriétaire...) cassaient silencieusement,
  ce qui empêchait la Facture Propriétaire de remonter le CA, le taux de
  commission MG Hôte, etc.
</commit_message>
<xml_diff>
--- a/gestion-mg-hote/MG_Hote_Gestion.xlsx
+++ b/gestion-mg-hote/MG_Hote_Gestion.xlsx
@@ -21,7 +21,7 @@
     <sheet name="Paramètres" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="Liste_Biens">Paramètres!$B$3:$B$12</definedName>
+    <definedName name="Liste_Biens">Biens!$A$5:$A$14</definedName>
     <definedName name="Liste_BiensGeneral">Paramètres!$C$3:$C$13</definedName>
     <definedName name="Liste_Plateformes">Paramètres!$D$3:$D$5</definedName>
     <definedName name="Liste_StatutResa">Paramètres!$E$3:$E$6</definedName>
@@ -1503,7 +1503,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="28">
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="F10:G10"/>
@@ -1880,7 +1880,7 @@
     <row r="34"/>
     <row r="35"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="31">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="G21:H21"/>
@@ -2213,7 +2213,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="42">
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A8:D8"/>
@@ -2365,15 +2365,13 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="38" t="inlineStr">
-        <is>
-          <t>Bien 1</t>
-        </is>
-      </c>
-      <c r="C3" s="38" t="inlineStr">
-        <is>
-          <t>Bien 1</t>
-        </is>
+      <c r="B3" s="38">
+        <f>IF(Biens!A5="","",Biens!A5)</f>
+        <v/>
+      </c>
+      <c r="C3" s="38">
+        <f>IF(Biens!A5="","",Biens!A5)</f>
+        <v/>
       </c>
       <c r="D3" s="38" t="inlineStr">
         <is>
@@ -2432,15 +2430,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="38" t="inlineStr">
-        <is>
-          <t>Bien 2</t>
-        </is>
-      </c>
-      <c r="C4" s="38" t="inlineStr">
-        <is>
-          <t>Bien 2</t>
-        </is>
+      <c r="B4" s="38">
+        <f>IF(Biens!A6="","",Biens!A6)</f>
+        <v/>
+      </c>
+      <c r="C4" s="38">
+        <f>IF(Biens!A6="","",Biens!A6)</f>
+        <v/>
       </c>
       <c r="D4" s="38" t="inlineStr">
         <is>
@@ -2499,15 +2495,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="38" t="inlineStr">
-        <is>
-          <t>Bien 3</t>
-        </is>
-      </c>
-      <c r="C5" s="38" t="inlineStr">
-        <is>
-          <t>Bien 3</t>
-        </is>
+      <c r="B5" s="38">
+        <f>IF(Biens!A7="","",Biens!A7)</f>
+        <v/>
+      </c>
+      <c r="C5" s="38">
+        <f>IF(Biens!A7="","",Biens!A7)</f>
+        <v/>
       </c>
       <c r="D5" s="38" t="inlineStr">
         <is>
@@ -2551,15 +2545,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="38" t="inlineStr">
-        <is>
-          <t>Bien 4</t>
-        </is>
-      </c>
-      <c r="C6" s="38" t="inlineStr">
-        <is>
-          <t>Bien 4</t>
-        </is>
+      <c r="B6" s="38">
+        <f>IF(Biens!A8="","",Biens!A8)</f>
+        <v/>
+      </c>
+      <c r="C6" s="38">
+        <f>IF(Biens!A8="","",Biens!A8)</f>
+        <v/>
       </c>
       <c r="E6" s="38" t="inlineStr">
         <is>
@@ -2583,15 +2575,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="38" t="inlineStr">
-        <is>
-          <t>Bien 5</t>
-        </is>
-      </c>
-      <c r="C7" s="38" t="inlineStr">
-        <is>
-          <t>Bien 5</t>
-        </is>
+      <c r="B7" s="38">
+        <f>IF(Biens!A9="","",Biens!A9)</f>
+        <v/>
+      </c>
+      <c r="C7" s="38">
+        <f>IF(Biens!A9="","",Biens!A9)</f>
+        <v/>
       </c>
       <c r="L7" s="38" t="inlineStr">
         <is>
@@ -2605,15 +2595,13 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="38" t="inlineStr">
-        <is>
-          <t>Bien 6</t>
-        </is>
-      </c>
-      <c r="C8" s="38" t="inlineStr">
-        <is>
-          <t>Bien 6</t>
-        </is>
+      <c r="B8" s="38">
+        <f>IF(Biens!A10="","",Biens!A10)</f>
+        <v/>
+      </c>
+      <c r="C8" s="38">
+        <f>IF(Biens!A10="","",Biens!A10)</f>
+        <v/>
       </c>
       <c r="L8" s="38" t="inlineStr">
         <is>
@@ -2622,15 +2610,13 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="38" t="inlineStr">
-        <is>
-          <t>Bien 7</t>
-        </is>
-      </c>
-      <c r="C9" s="38" t="inlineStr">
-        <is>
-          <t>Bien 7</t>
-        </is>
+      <c r="B9" s="38">
+        <f>IF(Biens!A11="","",Biens!A11)</f>
+        <v/>
+      </c>
+      <c r="C9" s="38">
+        <f>IF(Biens!A11="","",Biens!A11)</f>
+        <v/>
       </c>
       <c r="L9" s="38" t="inlineStr">
         <is>
@@ -2639,15 +2625,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="38" t="inlineStr">
-        <is>
-          <t>Bien 8</t>
-        </is>
-      </c>
-      <c r="C10" s="38" t="inlineStr">
-        <is>
-          <t>Bien 8</t>
-        </is>
+      <c r="B10" s="38">
+        <f>IF(Biens!A12="","",Biens!A12)</f>
+        <v/>
+      </c>
+      <c r="C10" s="38">
+        <f>IF(Biens!A12="","",Biens!A12)</f>
+        <v/>
       </c>
       <c r="L10" s="38" t="inlineStr">
         <is>
@@ -2656,15 +2640,13 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="38" t="inlineStr">
-        <is>
-          <t>Bien 9</t>
-        </is>
-      </c>
-      <c r="C11" s="38" t="inlineStr">
-        <is>
-          <t>Bien 9</t>
-        </is>
+      <c r="B11" s="38">
+        <f>IF(Biens!A13="","",Biens!A13)</f>
+        <v/>
+      </c>
+      <c r="C11" s="38">
+        <f>IF(Biens!A13="","",Biens!A13)</f>
+        <v/>
       </c>
       <c r="L11" s="38" t="inlineStr">
         <is>
@@ -2673,15 +2655,13 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="38" t="inlineStr">
-        <is>
-          <t>Bien 10</t>
-        </is>
-      </c>
-      <c r="C12" s="38" t="inlineStr">
-        <is>
-          <t>Bien 10</t>
-        </is>
+      <c r="B12" s="38">
+        <f>IF(Biens!A14="","",Biens!A14)</f>
+        <v/>
+      </c>
+      <c r="C12" s="38">
+        <f>IF(Biens!A14="","",Biens!A14)</f>
+        <v/>
       </c>
       <c r="L12" s="38" t="inlineStr">
         <is>
@@ -2702,7 +2682,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3095,7 +3075,7 @@
     <row r="77"/>
     <row r="78"/>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="44">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A43:H45"/>
@@ -11311,7 +11291,7 @@
       <c r="T204" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <autoFilter ref="A4:T204"/>
   <mergeCells count="4">
     <mergeCell ref="A1:B2"/>
@@ -11617,16 +11597,13 @@
       <c r="L14" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="C1:L1"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="A5:A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Liste_Biens</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation sqref="B5:B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Liste_TypeBien</formula1>
     </dataValidation>
@@ -11885,7 +11862,7 @@
       <c r="J14" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="C1:J1"/>
@@ -16500,7 +16477,7 @@
       <c r="J304" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <autoFilter ref="A4:J304"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B2"/>
@@ -17358,7 +17335,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
   <mergeCells count="4">
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A3:D3"/>
@@ -19433,7 +19410,7 @@
       <c r="K154" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <autoFilter ref="A4:K154"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B2"/>
@@ -20756,7 +20733,7 @@
       <c r="J104" s="26" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="0" password="C7B6"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0" password="C7B6"/>
   <autoFilter ref="A4:J104"/>
   <mergeCells count="3">
     <mergeCell ref="A1:B2"/>

</xml_diff>

<commit_message>
Facture Propriétaire : calcule le CA et la commission depuis Réservations
Le détail financier de la Facture Propriétaire ne recalcule plus le chiffre
d'affaires et la commission MG Hôte à partir d'une saisie manuelle dupliquée
dans le Journal Financier : il agrège désormais directement, par bien et par
période, les colonnes déjà calculées dans l'onglet Réservations (Prix total,
Frais plateforme, Montant net, Commission MG Hôte). Le détail affiche
maintenant la cascade complète (CA brut -> frais plateforme -> montant net
-> commission -> montant net à verser). Seules les charges refacturées
(Maintenance, Consommables, Électricité, Eau, Publicité) restent issues du
Journal Financier, ces dépenses n'étant pas rattachées à une réservation.
</commit_message>
<xml_diff>
--- a/gestion-mg-hote/MG_Hote_Gestion.xlsx
+++ b/gestion-mg-hote/MG_Hote_Gestion.xlsx
@@ -39,7 +39,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Synthèse Mensuelle'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Ménage'!$A$4:$K$154</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Maintenance'!$A$4:$J$104</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Facture Propriétaire'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Facture Propriétaire'!$A$1:$H$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'Rapport Mensuel'!$A$1:$F$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1563,7 +1563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1720,11 +1720,11 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="39" t="inlineStr">
         <is>
-          <t>Total recettes brutes (plateformes)</t>
+          <t>Chiffre d'affaires brut des réservations (Prix total)</t>
         </is>
       </c>
       <c r="G15" s="32">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Recette",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS(Réservations!$L$5:$L$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H15" s="40" t="n"/>
@@ -1732,23 +1732,23 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="38" t="inlineStr">
         <is>
-          <t>Taux de commission MG Hôte</t>
-        </is>
-      </c>
-      <c r="G16" s="34">
-        <f>IFERROR(INDEX(Biens!$I$5:$I$14,MATCH($G$5,Biens!$A$5:$A$14,0)),0)</f>
+          <t>Frais plateforme (Airbnb / Booking)</t>
+        </is>
+      </c>
+      <c r="G16" s="31">
+        <f>SUMIFS(Réservations!$M$5:$M$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H16" s="40" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="38" t="inlineStr">
-        <is>
-          <t>Montant commission MG Hôte</t>
-        </is>
-      </c>
-      <c r="G17" s="31">
-        <f>G15*G16</f>
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>Montant net après frais plateforme</t>
+        </is>
+      </c>
+      <c r="G17" s="32">
+        <f>SUMIFS(Réservations!$N$5:$N$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H17" s="40" t="n"/>
@@ -1756,11 +1756,11 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="38" t="inlineStr">
         <is>
-          <t>Charges refacturées au propriétaire :</t>
-        </is>
-      </c>
-      <c r="G18" s="28">
-        <f>""</f>
+          <t>Taux de commission MG Hôte</t>
+        </is>
+      </c>
+      <c r="G18" s="34">
+        <f>IFERROR(INDEX(Biens!$I$5:$I$14,MATCH($G$5,Biens!$A$5:$A$14,0)),0)</f>
         <v/>
       </c>
       <c r="H18" s="40" t="n"/>
@@ -1768,11 +1768,11 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Maintenance</t>
+          <t>Montant commission MG Hôte</t>
         </is>
       </c>
       <c r="G19" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Maintenance",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS(Réservations!$O$5:$O$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H19" s="40" t="n"/>
@@ -1780,11 +1780,11 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Consommables</t>
-        </is>
-      </c>
-      <c r="G20" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Consommables",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+          <t>Charges refacturées au propriétaire :</t>
+        </is>
+      </c>
+      <c r="G20" s="28">
+        <f>""</f>
         <v/>
       </c>
       <c r="H20" s="40" t="n"/>
@@ -1792,11 +1792,11 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Électricité</t>
+          <t xml:space="preserve">      Maintenance</t>
         </is>
       </c>
       <c r="G21" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Électricité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Maintenance",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
         <v/>
       </c>
       <c r="H21" s="40" t="n"/>
@@ -1804,11 +1804,11 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Eau</t>
+          <t xml:space="preserve">      Consommables</t>
         </is>
       </c>
       <c r="G22" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Eau",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Consommables",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
         <v/>
       </c>
       <c r="H22" s="40" t="n"/>
@@ -1816,76 +1816,103 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="38" t="inlineStr">
         <is>
+          <t xml:space="preserve">      Électricité</t>
+        </is>
+      </c>
+      <c r="G23" s="31">
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Électricité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <v/>
+      </c>
+      <c r="H23" s="40" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Eau</t>
+        </is>
+      </c>
+      <c r="G24" s="31">
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Eau",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <v/>
+      </c>
+      <c r="H24" s="40" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
           <t xml:space="preserve">      Publicité</t>
         </is>
       </c>
-      <c r="G23" s="31">
+      <c r="G25" s="31">
         <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Publicité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
         <v/>
       </c>
-      <c r="H23" s="40" t="n"/>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="39" t="inlineStr">
+      <c r="H25" s="40" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="39" t="inlineStr">
         <is>
           <t>Sous-total charges refacturées</t>
         </is>
       </c>
-      <c r="G24" s="32">
-        <f>SUM(G19:G23)</f>
-        <v/>
-      </c>
-      <c r="H24" s="40" t="n"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="G26" s="32">
+        <f>SUM(G21:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="40" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
         <is>
           <t>MONTANT NET À VERSER AU PROPRIÉTAIRE</t>
         </is>
       </c>
-      <c r="G25" s="42">
-        <f>G15-G17-G24</f>
-        <v/>
-      </c>
-      <c r="H25" s="40" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="G27" s="42">
+        <f>G17-G19-G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="40" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>Fait à ______________________, le</t>
         </is>
       </c>
-      <c r="D28" s="43">
+      <c r="D30" s="43">
         <f>TODAY()</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="44" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="44" t="inlineStr">
         <is>
           <t>Signature MG Hôte</t>
         </is>
       </c>
-      <c r="E31" s="44" t="inlineStr">
+      <c r="E33" s="44" t="inlineStr">
         <is>
           <t>Signature Propriétaire</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="45" t="n"/>
-      <c r="E32" s="45" t="n"/>
-    </row>
-    <row r="33"/>
-    <row r="34"/>
+    <row r="34">
+      <c r="A34" s="45" t="n"/>
+      <c r="E34" s="45" t="n"/>
+    </row>
     <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="C7B6"/>
-  <mergeCells count="31">
+  <mergeCells count="35">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="G21:H21"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="G27:H27"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="G23:H23"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="C2:H2"/>
@@ -1894,9 +1921,9 @@
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A17:F17"/>
+    <mergeCell ref="E34:H37"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="G18:H18"/>
-    <mergeCell ref="A32:D35"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="G24:H24"/>
     <mergeCell ref="G15:H15"/>
@@ -1904,11 +1931,12 @@
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="E32:H35"/>
+    <mergeCell ref="G26:H26"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="G25:H25"/>
+    <mergeCell ref="A34:D37"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="A25:F25"/>

</xml_diff>

<commit_message>
Corrige le CA à 0 sur Facture Propriétaire quand la période n'est pas remplie
Les cases "Période - du/au" étaient vides par défaut. Or dans les formules
SUMIFS, ">="&C6 / "<="&G6 avec une cellule vide se réduisent à ">="/"<=" que
Excel interprète comme ">=0"/"<=0" : la borne "<=0" excluait alors toutes les
vraies dates, donc le CA, les frais plateforme, le montant net et la
commission MG Hôte affichaient systématiquement 0 tant que la période
n'était pas saisie.

- Les formules ignorent maintenant une borne de période laissée vide au lieu
  de l'interpréter comme 0.
- "Période - du/au" est pré-rempli sur le mois en cours par défaut (comme
  sur Rapport Mensuel), pour que la facture affiche des chiffres dès
  l'ouverture du fichier.
</commit_message>
<xml_diff>
--- a/gestion-mg-hote/MG_Hote_Gestion.xlsx
+++ b/gestion-mg-hote/MG_Hote_Gestion.xlsx
@@ -892,6 +892,21 @@
     <author>MG Hôte</author>
   </authors>
   <commentList>
+    <comment ref="C6" authorId="0" shapeId="0">
+      <text>
+        <t>Pré-rempli sur le mois en cours. Remplacez par une vraie date (pas une formule) pour figer la période de cette facture.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>MG Hôte</author>
+  </authors>
+  <commentList>
     <comment ref="D4" authorId="0" shapeId="0">
       <text>
         <t>Saisissez le 1er jour du mois à analyser (ex: 01/07/2026). Toutes les données ci-dessous se recalculent automatiquement.</t>
@@ -1637,13 +1652,19 @@
           <t>Période — du</t>
         </is>
       </c>
-      <c r="C6" s="27" t="n"/>
+      <c r="C6" s="27">
+        <f>EOMONTH(TODAY(),-1)+1</f>
+        <v/>
+      </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
           <t>au</t>
         </is>
       </c>
-      <c r="G6" s="27" t="n"/>
+      <c r="G6" s="27">
+        <f>EOMONTH(TODAY(),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -1724,7 +1745,7 @@
         </is>
       </c>
       <c r="G15" s="32">
-        <f>SUMIFS(Réservations!$L$5:$L$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
+        <f>SUMIFS(Réservations!$L$5:$L$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;IF($C$6="",0,$C$6),Réservations!$G$5:$G$204,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6),Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H15" s="40" t="n"/>
@@ -1736,7 +1757,7 @@
         </is>
       </c>
       <c r="G16" s="31">
-        <f>SUMIFS(Réservations!$M$5:$M$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
+        <f>SUMIFS(Réservations!$M$5:$M$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;IF($C$6="",0,$C$6),Réservations!$G$5:$G$204,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6),Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H16" s="40" t="n"/>
@@ -1748,7 +1769,7 @@
         </is>
       </c>
       <c r="G17" s="32">
-        <f>SUMIFS(Réservations!$N$5:$N$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
+        <f>SUMIFS(Réservations!$N$5:$N$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;IF($C$6="",0,$C$6),Réservations!$G$5:$G$204,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6),Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H17" s="40" t="n"/>
@@ -1772,7 +1793,7 @@
         </is>
       </c>
       <c r="G19" s="31">
-        <f>SUMIFS(Réservations!$O$5:$O$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;$C$6,Réservations!$G$5:$G$204,"&lt;="&amp;$G$6,Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
+        <f>SUMIFS(Réservations!$O$5:$O$204,Réservations!$B$5:$B$204,$G$5,Réservations!$G$5:$G$204,"&gt;="&amp;IF($C$6="",0,$C$6),Réservations!$G$5:$G$204,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6),Réservations!$Q$5:$Q$204,"&lt;&gt;Annulée")</f>
         <v/>
       </c>
       <c r="H19" s="40" t="n"/>
@@ -1796,7 +1817,7 @@
         </is>
       </c>
       <c r="G21" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Maintenance",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Maintenance",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;IF($C$6="",0,$C$6),'Journal Financier'!$A$5:$A$304,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6))</f>
         <v/>
       </c>
       <c r="H21" s="40" t="n"/>
@@ -1808,7 +1829,7 @@
         </is>
       </c>
       <c r="G22" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Consommables",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Consommables",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;IF($C$6="",0,$C$6),'Journal Financier'!$A$5:$A$304,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6))</f>
         <v/>
       </c>
       <c r="H22" s="40" t="n"/>
@@ -1820,7 +1841,7 @@
         </is>
       </c>
       <c r="G23" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Électricité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Électricité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;IF($C$6="",0,$C$6),'Journal Financier'!$A$5:$A$304,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6))</f>
         <v/>
       </c>
       <c r="H23" s="40" t="n"/>
@@ -1832,7 +1853,7 @@
         </is>
       </c>
       <c r="G24" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Eau",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Eau",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;IF($C$6="",0,$C$6),'Journal Financier'!$A$5:$A$304,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6))</f>
         <v/>
       </c>
       <c r="H24" s="40" t="n"/>
@@ -1844,7 +1865,7 @@
         </is>
       </c>
       <c r="G25" s="31">
-        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Publicité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;$C$6,'Journal Financier'!$A$5:$A$304,"&lt;="&amp;$G$6)</f>
+        <f>SUMIFS('Journal Financier'!$F$5:$F$304,'Journal Financier'!$B$5:$B$304,$G$5,'Journal Financier'!$C$5:$C$304,"Dépense",'Journal Financier'!$D$5:$D$304,"Publicité",'Journal Financier'!$A$5:$A$304,"&gt;="&amp;IF($C$6="",0,$C$6),'Journal Financier'!$A$5:$A$304,"&lt;="&amp;IF($G$6="",DATE(2099,12,31),$G$6))</f>
         <v/>
       </c>
       <c r="H25" s="40" t="n"/>
@@ -1949,6 +1970,7 @@
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>